<commit_message>
Fix Supabase pooler crash on startup
</commit_message>
<xml_diff>
--- a/frontend/snapshot/api/workbook.xlsx
+++ b/frontend/snapshot/api/workbook.xlsx
@@ -576,7 +576,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Greenlight Robotics Inc.</t>
+          <t>Tianzheng Biotechnology Inc</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -586,7 +586,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Robotics &amp; Physical AI</t>
+          <t>BioTech &amp; Health AI</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -629,17 +629,17 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>100th pct of 12 in robotics|unknown (low-confidence cohort &lt;20)</t>
+          <t>100th pct of 6 in biotech_health|unknown (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>robotics</t>
+          <t>biotech_health</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -649,7 +649,7 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>briefs/greenlight-robotics-inc.md</t>
+          <t>briefs/tianzheng-biotechnology-inc.md</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -661,7 +661,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Tianzheng Biotechnology Inc</t>
+          <t>Global Defense, Inc.</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -671,7 +671,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>BioTech &amp; Health AI</t>
+          <t>Defence Tech</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -714,39 +714,39 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>100th pct of 4 in biotech_health|unknown (low-confidence cohort &lt;20)</t>
+          <t>100th pct of 2 in defence_tech|unknown (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>biotech_health</t>
+          <t>defence_tech</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Deep Dive</t>
+          <t>Watch</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>briefs/tianzheng-biotechnology-inc.md</t>
+          <t>briefs/global-defense-inc.md</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>— (no commentary captured yet; X/Blind/podcasts require licenses)</t>
+          <t>10 items; latest: Defense industry is a small fraction of the notebook market, meaning Lenovo is s…</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Global Defense, Inc.</t>
+          <t>Greenlight Robotics Inc.</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -756,7 +756,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Defence Tech</t>
+          <t>Robotics &amp; Physical AI</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -799,32 +799,32 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>100th pct of 2 in defence_tech|unknown (low-confidence cohort &lt;20)</t>
+          <t>100th pct of 15 in robotics|unknown (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>defence_tech</t>
+          <t>robotics</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Watch</t>
+          <t>Deep Dive</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>briefs/global-defense-inc.md</t>
+          <t>briefs/greenlight-robotics-inc.md</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>10 items; latest: Defense industry is a small fraction of the notebook market, meaning Lenovo is s…</t>
+          <t>— (no commentary captured yet; X/Blind/podcasts require licenses)</t>
         </is>
       </c>
     </row>
@@ -884,7 +884,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>100th pct of 10 in unclassified|unknown (low-confidence cohort &lt;20)</t>
+          <t>100th pct of 11 in unclassified|unknown (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -969,7 +969,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>100th pct of 4 in unclassified|series-b (low-confidence cohort &lt;20)</t>
+          <t>100th pct of 5 in unclassified|series-b (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -1054,7 +1054,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>92th pct of 12 in robotics|unknown (low-confidence cohort &lt;20)</t>
+          <t>93th pct of 15 in robotics|unknown (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>90th pct of 10 in unclassified|unknown (low-confidence cohort &lt;20)</t>
+          <t>91th pct of 11 in unclassified|unknown (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>83th pct of 12 in robotics|unknown (low-confidence cohort &lt;20)</t>
+          <t>87th pct of 15 in robotics|unknown (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1256,7 +1256,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Tech-Infused Pool Hall Startup</t>
+          <t>Los Angeles Project Inc</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1266,7 +1266,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>unclassified</t>
+          <t>BioTech &amp; Health AI</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1276,12 +1276,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>$55.0M</t>
+          <t>— (not disclosed in free sources)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1309,17 +1309,17 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>80th pct of 10 in unclassified|unknown (low-confidence cohort &lt;20)</t>
+          <t>83th pct of 6 in biotech_health|unknown (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>biotech_health</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -1341,7 +1341,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>WALDEN ROBOTICS, INC.</t>
+          <t>Tech-Infused Pool Hall Startup</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1351,7 +1351,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Robotics &amp; Physical AI</t>
+          <t>unclassified</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1361,12 +1361,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>— (not disclosed in free sources)</t>
+          <t>$55.0M</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1394,17 +1394,17 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>75th pct of 12 in robotics|unknown (low-confidence cohort &lt;20)</t>
+          <t>82th pct of 11 in unclassified|unknown (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>robotics</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
@@ -1426,7 +1426,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Los Angeles Project Inc</t>
+          <t>Dust</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1436,22 +1436,22 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>BioTech &amp; Health AI</t>
+          <t>unclassified</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>series-b</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>— (not disclosed in free sources)</t>
+          <t>$40.0M</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1479,17 +1479,17 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>75th pct of 4 in biotech_health|unknown (low-confidence cohort &lt;20)</t>
+          <t>80th pct of 5 in unclassified|series-b (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>biotech_health</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
@@ -1511,7 +1511,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Dust</t>
+          <t>WALDEN ROBOTICS, INC.</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1521,22 +1521,22 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>unclassified</t>
+          <t>Robotics &amp; Physical AI</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>series-b</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>$40.0M</t>
+          <t>— (not disclosed in free sources)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1564,17 +1564,17 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>75th pct of 4 in unclassified|series-b (low-confidence cohort &lt;20)</t>
+          <t>80th pct of 15 in robotics|unknown (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>robotics</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
@@ -1596,7 +1596,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Moonshot AI</t>
+          <t>Halcyon Robotics Corp</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1606,7 +1606,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>unclassified</t>
+          <t>Robotics &amp; Physical AI</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1616,12 +1616,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>$3.50B</t>
+          <t>— (not disclosed in free sources)</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1649,17 +1649,17 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>70th pct of 10 in unclassified|unknown (low-confidence cohort &lt;20)</t>
+          <t>73th pct of 15 in robotics|unknown (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>robotics</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
@@ -1681,7 +1681,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Halcyon Robotics Corp</t>
+          <t>Moonshot AI</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1691,7 +1691,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Robotics &amp; Physical AI</t>
+          <t>unclassified</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1701,12 +1701,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>— (not disclosed in free sources)</t>
+          <t>$3.50B</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1734,17 +1734,17 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>67th pct of 12 in robotics|unknown (low-confidence cohort &lt;20)</t>
+          <t>73th pct of 11 in unclassified|unknown (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>robotics</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
@@ -1766,7 +1766,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Travis Kalanick's Atoms</t>
+          <t>Portal Biotechnologies, Inc.</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1776,7 +1776,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>unclassified</t>
+          <t>BioTech &amp; Health AI</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1786,12 +1786,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>$1.70B</t>
+          <t>— (not disclosed in free sources)</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1819,17 +1819,17 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>60th pct of 10 in unclassified|unknown (low-confidence cohort &lt;20)</t>
+          <t>67th pct of 6 in biotech_health|unknown (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>biotech_health</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
@@ -1851,7 +1851,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>JuliaHub</t>
+          <t>NEURA Robotics Moonrock Cap Ltd</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1861,22 +1861,22 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>unclassified</t>
+          <t>Robotics &amp; Physical AI</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>series-b</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$65.0M</t>
+          <t>— (not disclosed in free sources)</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1904,17 +1904,17 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>60th pct of 5 in unclassified|series-b (low-confidence cohort &lt;20)</t>
+          <t>67th pct of 15 in robotics|unknown (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>robotics</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
@@ -1936,7 +1936,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>NEURA Robotics Moonrock Cap Ltd</t>
+          <t>Travis Kalanick's Atoms</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1946,7 +1946,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Robotics &amp; Physical AI</t>
+          <t>unclassified</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1956,12 +1956,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>— (not disclosed in free sources)</t>
+          <t>$1.70B</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1989,17 +1989,17 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>58th pct of 12 in robotics|unknown (low-confidence cohort &lt;20)</t>
+          <t>64th pct of 11 in unclassified|unknown (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>robotics</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
@@ -2021,7 +2021,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Antares Nuclear, Inc.</t>
+          <t>Fleet Robotics, Inc.</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2031,7 +2031,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Energy-as-a-service</t>
+          <t>Robotics &amp; Physical AI</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -2074,22 +2074,22 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>50th pct of 1 in energy|unknown (low-confidence cohort &lt;20)</t>
+          <t>60th pct of 15 in robotics|unknown (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>energy</t>
+          <t>robotics</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Watch</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
@@ -2106,7 +2106,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Askari Defense, Inc.</t>
+          <t>JuliaHub</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2116,22 +2116,22 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Defence Tech</t>
+          <t>unclassified</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>series-b</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>— (not disclosed in free sources)</t>
+          <t>$65.0M</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -2159,22 +2159,22 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>50th pct of 2 in defence_tech|unknown (low-confidence cohort &lt;20)</t>
+          <t>60th pct of 5 in unclassified|series-b (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>defence_tech</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Watch</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
@@ -2244,7 +2244,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>50th pct of 10 in unclassified|unknown (low-confidence cohort &lt;20)</t>
+          <t>54th pct of 11 in unclassified|unknown (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -2276,7 +2276,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Fleet Robotics, Inc.</t>
+          <t>Unleashed Robotics, Inc.</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2329,7 +2329,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>50th pct of 12 in robotics|unknown (low-confidence cohort &lt;20)</t>
+          <t>53th pct of 15 in robotics|unknown (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -2344,7 +2344,7 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>Watch</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
@@ -2361,7 +2361,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Portal Biotechnologies, Inc.</t>
+          <t>Sitrep</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2371,7 +2371,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>BioTech &amp; Health AI</t>
+          <t>AI in manufacturing / AI copilots</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -2414,22 +2414,22 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>50th pct of 4 in biotech_health|unknown (low-confidence cohort &lt;20)</t>
+          <t>50th pct of 1 in ai_manufacturing|unknown (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>biotech_health</t>
+          <t>ai_manufacturing</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>Watch</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
@@ -2446,7 +2446,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Augustus</t>
+          <t>Askari Defense, Inc.</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2456,7 +2456,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Fintech &amp; Financial Infrastructure</t>
+          <t>Defence Tech</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -2466,12 +2466,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>$180.0M</t>
+          <t>— (not disclosed in free sources)</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -2499,17 +2499,17 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>50th pct of 1 in fintech|unknown (low-confidence cohort &lt;20)</t>
+          <t>50th pct of 2 in defence_tech|unknown (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>fintech</t>
+          <t>defence_tech</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
@@ -2531,7 +2531,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>OpenRouter</t>
+          <t>Thea Energy</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2541,7 +2541,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>unclassified</t>
+          <t>AI Infrastructure &amp; Compute Stack</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2551,12 +2551,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>$113.0M</t>
+          <t>$100.0M</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -2584,17 +2584,17 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>50th pct of 4 in unclassified|series-b (low-confidence cohort &lt;20)</t>
+          <t>50th pct of 1 in ai_infrastructure|series-b (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ai_infrastructure</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
@@ -2616,7 +2616,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Thea Energy</t>
+          <t>Cyrus Biotechnology, Inc.</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2626,22 +2626,22 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>AI Infrastructure &amp; Compute Stack</t>
+          <t>BioTech &amp; Health AI</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>series-b</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>$100.0M</t>
+          <t>— (not disclosed in free sources)</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -2669,17 +2669,17 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>50th pct of 1 in ai_infrastructure|series-b (low-confidence cohort &lt;20)</t>
+          <t>50th pct of 6 in biotech_health|unknown (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>ai_infrastructure</t>
+          <t>biotech_health</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
@@ -2701,7 +2701,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Sitrep</t>
+          <t>Antares Nuclear, Inc.</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2711,7 +2711,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>AI in manufacturing / AI copilots</t>
+          <t>Energy-as-a-service</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2754,17 +2754,17 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>50th pct of 1 in ai_manufacturing|unknown (low-confidence cohort &lt;20)</t>
+          <t>50th pct of 1 in energy|unknown (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>ai_manufacturing</t>
+          <t>energy</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
@@ -2786,7 +2786,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Unleashed Robotics, Inc.</t>
+          <t>Augustus</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2796,7 +2796,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Robotics &amp; Physical AI</t>
+          <t>Fintech &amp; Financial Infrastructure</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2806,12 +2806,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>— (not disclosed in free sources)</t>
+          <t>$180.0M</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -2839,17 +2839,17 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>42th pct of 12 in robotics|unknown (low-confidence cohort &lt;20)</t>
+          <t>50th pct of 1 in fintech|unknown (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>robotics</t>
+          <t>fintech</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="O28" t="inlineStr">
@@ -2871,7 +2871,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Artificial Intelligence Financial Services Market Inc.</t>
+          <t>Bird's Eye Robotics, Inc.</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2881,7 +2881,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>unclassified</t>
+          <t>Robotics &amp; Physical AI</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2924,17 +2924,17 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>40th pct of 10 in unclassified|unknown (low-confidence cohort &lt;20)</t>
+          <t>47th pct of 15 in robotics|unknown (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>robotics</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
@@ -2956,7 +2956,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Bird's Eye Robotics, Inc.</t>
+          <t>Artificial Intelligence Financial Services Market Inc.</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2966,7 +2966,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Robotics &amp; Physical AI</t>
+          <t>unclassified</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -3009,17 +3009,17 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>33th pct of 12 in robotics|unknown (low-confidence cohort &lt;20)</t>
+          <t>46th pct of 11 in unclassified|unknown (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>robotics</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
@@ -3041,7 +3041,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Mentat Biotechnology, Corp.</t>
+          <t>AMP Robotics Corp</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3051,7 +3051,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>BioTech &amp; Health AI</t>
+          <t>Robotics &amp; Physical AI</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -3094,17 +3094,17 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>33th pct of 6 in biotech_health|unknown (low-confidence cohort &lt;20)</t>
+          <t>40th pct of 15 in robotics|unknown (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>biotech_health</t>
+          <t>robotics</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
@@ -3126,7 +3126,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Panorama Artificial Intelligence Corp.</t>
+          <t>OpenRouter</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -3141,17 +3141,17 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>series-b</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>— (not disclosed in free sources)</t>
+          <t>$113.0M</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -3179,7 +3179,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>30th pct of 10 in unclassified|unknown (low-confidence cohort &lt;20)</t>
+          <t>40th pct of 5 in unclassified|series-b (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -3189,7 +3189,7 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
@@ -3211,7 +3211,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>AMP Robotics Corp</t>
+          <t>Panorama Artificial Intelligence Corp.</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3221,7 +3221,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Robotics &amp; Physical AI</t>
+          <t>unclassified</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -3264,17 +3264,17 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>25th pct of 12 in robotics|unknown (low-confidence cohort &lt;20)</t>
+          <t>36th pct of 11 in unclassified|unknown (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>robotics</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
@@ -3296,7 +3296,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Cyrus Biotechnology, Inc.</t>
+          <t>CHANNEL ROBOTICS, INC.</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -3306,7 +3306,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>BioTech &amp; Health AI</t>
+          <t>Robotics &amp; Physical AI</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -3349,17 +3349,17 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>25th pct of 4 in biotech_health|unknown (low-confidence cohort &lt;20)</t>
+          <t>33th pct of 15 in robotics|unknown (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>biotech_health</t>
+          <t>robotics</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="O34" t="inlineStr">
@@ -3381,7 +3381,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>DeepInfra</t>
+          <t>Mentat Biotechnology, Corp.</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -3391,22 +3391,22 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>unclassified</t>
+          <t>BioTech &amp; Health AI</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>series-b</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>$107.0M</t>
+          <t>— (not disclosed in free sources)</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -3434,17 +3434,17 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>25th pct of 4 in unclassified|series-b (low-confidence cohort &lt;20)</t>
+          <t>33th pct of 6 in biotech_health|unknown (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>biotech_health</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
@@ -3519,7 +3519,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>20th pct of 10 in unclassified|unknown (low-confidence cohort &lt;20)</t>
+          <t>27th pct of 11 in unclassified|unknown (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -3551,7 +3551,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CHANNEL ROBOTICS, INC.</t>
+          <t>Digital Intelligence Robotics Ltd</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -3604,7 +3604,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>17th pct of 12 in robotics|unknown (low-confidence cohort &lt;20)</t>
+          <t>27th pct of 15 in robotics|unknown (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -3614,7 +3614,7 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="O37" t="inlineStr">
@@ -3636,7 +3636,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Vitanova Biomedical Inc.</t>
+          <t>Pentra Robotics, inc.</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -3646,7 +3646,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>BioTech &amp; Health AI</t>
+          <t>Robotics &amp; Physical AI</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -3689,17 +3689,17 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>17th pct of 6 in biotech_health|unknown (low-confidence cohort &lt;20)</t>
+          <t>20th pct of 15 in robotics|unknown (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>biotech_health</t>
+          <t>robotics</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
@@ -3721,7 +3721,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Sielo Robotics Inc.</t>
+          <t>DeepInfra</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -3731,22 +3731,22 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Robotics &amp; Physical AI</t>
+          <t>unclassified</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>series-b</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>— (not disclosed in free sources)</t>
+          <t>$107.0M</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -3774,17 +3774,17 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>14th pct of 14 in robotics|unknown (low-confidence cohort &lt;20)</t>
+          <t>20th pct of 5 in unclassified|series-b (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>robotics</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
@@ -3859,7 +3859,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>10th pct of 10 in unclassified|unknown (low-confidence cohort &lt;20)</t>
+          <t>18th pct of 11 in unclassified|unknown (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
@@ -3891,7 +3891,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Venus Aerospace Corp.</t>
+          <t>Vitanova Biomedical Inc.</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -3901,7 +3901,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>unclassified</t>
+          <t>BioTech &amp; Health AI</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -3944,17 +3944,17 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>9th pct of 11 in unclassified|unknown (low-confidence cohort &lt;20)</t>
+          <t>17th pct of 6 in biotech_health|unknown (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>biotech_health</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="O41" t="inlineStr">
@@ -3976,7 +3976,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Digital Intelligence Robotics Ltd</t>
+          <t>Luminous Robotics, Inc.</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -4029,7 +4029,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>8th pct of 12 in robotics|unknown (low-confidence cohort &lt;20)</t>
+          <t>13th pct of 15 in robotics|unknown (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
@@ -4039,7 +4039,7 @@
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
@@ -4061,7 +4061,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Pentra Robotics, inc.</t>
+          <t>Venus Aerospace Corp.</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -4071,7 +4071,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Robotics &amp; Physical AI</t>
+          <t>unclassified</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -4114,17 +4114,17 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>7th pct of 14 in robotics|unknown (low-confidence cohort &lt;20)</t>
+          <t>9th pct of 11 in unclassified|unknown (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>robotics</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
@@ -4146,7 +4146,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Luminous Robotics, Inc.</t>
+          <t>Sielo Robotics Inc.</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -4209,7 +4209,7 @@
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="O44" t="inlineStr">
@@ -4314,7 +4314,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-07-30T06:14:11Z</t>
+          <t>2026-08-05T20:30:18Z</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -4346,7 +4346,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-07-30T06:14:01Z</t>
+          <t>2026-08-05T20:30:08Z</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -4442,7 +4442,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-07-30T06:14:01Z</t>
+          <t>2026-08-05T20:30:08Z</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -4506,7 +4506,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-07-30T06:14:11Z</t>
+          <t>2026-08-05T20:30:18Z</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -4538,7 +4538,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-07-30T06:14:11Z</t>
+          <t>2026-08-05T20:30:18Z</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -4570,7 +4570,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-07-30T06:14:11Z</t>
+          <t>2026-08-05T20:30:18Z</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -4602,7 +4602,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-07-30T06:14:11Z</t>
+          <t>2026-08-05T20:30:18Z</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -4634,7 +4634,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-07-30T06:14:11Z</t>
+          <t>2026-08-05T20:30:18Z</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -4819,7 +4819,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>last_signal_at=2026-04-21 (backdated 100d) -&gt; appears in Stale flow flagged for partner review; NOT deleted</t>
+          <t>last_signal_at=2026-04-27 (backdated 100d) -&gt; appears in Stale flow flagged for partner review; NOT deleted</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -4965,7 +4965,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Greenlight Robotics Inc.</t>
+          <t>Tianzheng Biotechnology Inc</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -4975,7 +4975,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Robotics &amp; Physical AI</t>
+          <t>BioTech &amp; Health AI</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -5018,17 +5018,17 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>100th pct of 12 in robotics|unknown (low-confidence cohort &lt;20)</t>
+          <t>100th pct of 6 in biotech_health|unknown (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>robotics</t>
+          <t>biotech_health</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -5038,7 +5038,7 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>briefs/greenlight-robotics-inc.md</t>
+          <t>briefs/tianzheng-biotechnology-inc.md</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -5050,7 +5050,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Tianzheng Biotechnology Inc</t>
+          <t>Greenlight Robotics Inc.</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -5060,7 +5060,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>BioTech &amp; Health AI</t>
+          <t>Robotics &amp; Physical AI</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -5103,17 +5103,17 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>100th pct of 4 in biotech_health|unknown (low-confidence cohort &lt;20)</t>
+          <t>100th pct of 15 in robotics|unknown (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>biotech_health</t>
+          <t>robotics</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -5123,7 +5123,7 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>briefs/tianzheng-biotechnology-inc.md</t>
+          <t>briefs/greenlight-robotics-inc.md</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
@@ -5188,7 +5188,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>100th pct of 10 in unclassified|unknown (low-confidence cohort &lt;20)</t>
+          <t>100th pct of 11 in unclassified|unknown (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -5273,7 +5273,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>92th pct of 12 in robotics|unknown (low-confidence cohort &lt;20)</t>
+          <t>93th pct of 15 in robotics|unknown (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -5358,7 +5358,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>90th pct of 10 in unclassified|unknown (low-confidence cohort &lt;20)</t>
+          <t>91th pct of 11 in unclassified|unknown (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -5443,7 +5443,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>83th pct of 12 in robotics|unknown (low-confidence cohort &lt;20)</t>
+          <t>87th pct of 15 in robotics|unknown (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -5694,7 +5694,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Tech-Infused Pool Hall Startup</t>
+          <t>Los Angeles Project Inc</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -5704,7 +5704,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>unclassified</t>
+          <t>BioTech &amp; Health AI</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -5714,12 +5714,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>$55.0M</t>
+          <t>— (not disclosed in free sources)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -5747,17 +5747,17 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>80th pct of 10 in unclassified|unknown (low-confidence cohort &lt;20)</t>
+          <t>83th pct of 6 in biotech_health|unknown (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>biotech_health</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -5779,7 +5779,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>WALDEN ROBOTICS, INC.</t>
+          <t>Tech-Infused Pool Hall Startup</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -5789,7 +5789,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Robotics &amp; Physical AI</t>
+          <t>unclassified</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -5799,12 +5799,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>— (not disclosed in free sources)</t>
+          <t>$55.0M</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -5832,17 +5832,17 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>75th pct of 12 in robotics|unknown (low-confidence cohort &lt;20)</t>
+          <t>82th pct of 11 in unclassified|unknown (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>robotics</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -5864,7 +5864,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Los Angeles Project Inc</t>
+          <t>Dust</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -5874,22 +5874,22 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>BioTech &amp; Health AI</t>
+          <t>unclassified</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>series-b</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>— (not disclosed in free sources)</t>
+          <t>$40.0M</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -5917,17 +5917,17 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>75th pct of 4 in biotech_health|unknown (low-confidence cohort &lt;20)</t>
+          <t>80th pct of 5 in unclassified|series-b (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>biotech_health</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -5949,7 +5949,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Dust</t>
+          <t>WALDEN ROBOTICS, INC.</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -5959,22 +5959,22 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>unclassified</t>
+          <t>Robotics &amp; Physical AI</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>series-b</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>$40.0M</t>
+          <t>— (not disclosed in free sources)</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -6002,17 +6002,17 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>75th pct of 4 in unclassified|series-b (low-confidence cohort &lt;20)</t>
+          <t>80th pct of 15 in robotics|unknown (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>robotics</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -6034,7 +6034,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Moonshot AI</t>
+          <t>Halcyon Robotics Corp</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -6044,7 +6044,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>unclassified</t>
+          <t>Robotics &amp; Physical AI</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -6054,12 +6054,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>$3.50B</t>
+          <t>— (not disclosed in free sources)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -6087,17 +6087,17 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>70th pct of 10 in unclassified|unknown (low-confidence cohort &lt;20)</t>
+          <t>73th pct of 15 in robotics|unknown (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>robotics</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -6119,7 +6119,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Halcyon Robotics Corp</t>
+          <t>Moonshot AI</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -6129,7 +6129,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Robotics &amp; Physical AI</t>
+          <t>unclassified</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -6139,12 +6139,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>— (not disclosed in free sources)</t>
+          <t>$3.50B</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -6172,17 +6172,17 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>67th pct of 12 in robotics|unknown (low-confidence cohort &lt;20)</t>
+          <t>73th pct of 11 in unclassified|unknown (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>robotics</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -6204,7 +6204,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Travis Kalanick's Atoms</t>
+          <t>Portal Biotechnologies, Inc.</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -6214,7 +6214,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>unclassified</t>
+          <t>BioTech &amp; Health AI</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -6224,12 +6224,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>$1.70B</t>
+          <t>— (not disclosed in free sources)</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -6257,17 +6257,17 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>60th pct of 10 in unclassified|unknown (low-confidence cohort &lt;20)</t>
+          <t>67th pct of 6 in biotech_health|unknown (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>biotech_health</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
@@ -6289,7 +6289,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>JuliaHub</t>
+          <t>NEURA Robotics Moonrock Cap Ltd</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -6299,22 +6299,22 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>unclassified</t>
+          <t>Robotics &amp; Physical AI</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>series-b</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>$65.0M</t>
+          <t>— (not disclosed in free sources)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -6342,17 +6342,17 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>60th pct of 5 in unclassified|series-b (low-confidence cohort &lt;20)</t>
+          <t>67th pct of 15 in robotics|unknown (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>robotics</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -6374,7 +6374,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>NEURA Robotics Moonrock Cap Ltd</t>
+          <t>Travis Kalanick's Atoms</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -6384,7 +6384,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Robotics &amp; Physical AI</t>
+          <t>unclassified</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -6394,12 +6394,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>— (not disclosed in free sources)</t>
+          <t>$1.70B</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -6427,17 +6427,17 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>58th pct of 12 in robotics|unknown (low-confidence cohort &lt;20)</t>
+          <t>64th pct of 11 in unclassified|unknown (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>robotics</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
@@ -6512,7 +6512,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>50th pct of 12 in robotics|unknown (low-confidence cohort &lt;20)</t>
+          <t>60th pct of 15 in robotics|unknown (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -6544,7 +6544,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Portal Biotechnologies, Inc.</t>
+          <t>JuliaHub</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -6554,22 +6554,22 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>BioTech &amp; Health AI</t>
+          <t>unclassified</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>series-b</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>— (not disclosed in free sources)</t>
+          <t>$65.0M</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -6597,17 +6597,17 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>50th pct of 4 in biotech_health|unknown (low-confidence cohort &lt;20)</t>
+          <t>60th pct of 5 in unclassified|series-b (low-confidence cohort &lt;20)</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>biotech_health</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
@@ -6646,7 +6646,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N7"/>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -6758,7 +6758,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -6768,7 +6768,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/2142598/000214259826000001/0002142598-26-000001-index.htm; https://www.sec.gov/Archives/edgar/data/2145725/000214572526000002/0002145725-26-000002-index.htm; https://www.sec.gov/Archives/edgar/data/2144409/000123191926000765/0001231919-26-000765-index.htm; https://www.sec.gov/Archives/edgar/data/2144337/000214433726000002/0002144337-26-000002-index.htm</t>
+          <t>https://www.sec.gov/Archives/edgar/data/2140567/000214056726000001/0002140567-26-000001-index.htm; https://www.sec.gov/Archives/edgar/data/2146041/000121390026081773/0001213900-26-081773-index.htm; https://www.sec.gov/Archives/edgar/data/2145832/000214583226000001/0002145832-26-000001-index.htm; https://www.sec.gov/Archives/edgar/data/2142598/000214259826000001/0002142598-26-000001-index.htm</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -6780,28 +6780,28 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>robotics</t>
+          <t>defense</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>robotics, cgf2021, master, gaingels, burlington, nonpublic</t>
+          <t>defense, dover, decimus, select, security, aventura</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="F3" t="n">
         <v>2</v>
       </c>
       <c r="G3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -6810,203 +6810,15 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Greenlight Robotics Inc. (100th pct, Deep Dive); Halcyon Robotics Corp (71th pct, Watch); Digital Intelligence Robotics Ltd (21th pct, Pass); Novara Robotics Inc. (86th pct, Deep Dive); WALDEN ROBOTICS, INC. (79th pct, Watch)</t>
+          <t>Global Defense, Inc. (100th pct, Deep Dive); Askari Defense, Inc. (50th pct, Pass); Mentat Biotechnology, Corp. (33th pct, Pass)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/2142598/000214259826000001/0002142598-26-000001-index.htm; https://www.sec.gov/Archives/edgar/data/2145725/000214572526000002/0002145725-26-000002-index.htm; https://www.sec.gov/Archives/edgar/data/2144409/000123191926000765/0001231919-26-000765-index.htm; https://www.sec.gov/Archives/edgar/data/2144337/000214433726000002/0002144337-26-000002-index.htm</t>
+          <t>https://www.sec.gov/Archives/edgar/data/2133514/000101297526000649/0001012975-26-000649-index.htm; https://www.sec.gov/Archives/edgar/data/2128641/000101297526000648/0001012975-26-000648-index.htm; https://www.sec.gov/Archives/edgar/data/2144303/000214430326000001/0002144303-26-000001-index.htm; https://www.sec.gov/Archives/edgar/data/2037822/000203782226000003/0002037822-26-000003-index.htm</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
-        <is>
-          <t>Emerging: technical signal running ahead of mainstream coverage.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>robotics</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>robotics, cgf2021, master, burlington, gaingels, nonpublic</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>9</v>
-      </c>
-      <c r="D4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E4" t="n">
-        <v>9</v>
-      </c>
-      <c r="F4" t="n">
-        <v>2</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>Greenlight Robotics Inc. (100th pct, Deep Dive); Halcyon Robotics Corp (67th pct, Watch); Digital Intelligence Robotics Ltd (8th pct, Pass); Novara Robotics Inc. (83th pct, Watch); WALDEN ROBOTICS, INC. (75th pct, Watch)</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/2142598/000214259826000001/0002142598-26-000001-index.htm; https://www.sec.gov/Archives/edgar/data/2145725/000214572526000002/0002145725-26-000002-index.htm; https://www.sec.gov/Archives/edgar/data/2144409/000123191926000765/0001231919-26-000765-index.htm; https://www.sec.gov/Archives/edgar/data/2144337/000214433726000002/0002144337-26-000002-index.htm</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>Emerging: technical signal running ahead of mainstream coverage.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>defense</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>defense, dover, decimus, select, security, aventura</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>12</v>
-      </c>
-      <c r="D5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" t="n">
-        <v>6</v>
-      </c>
-      <c r="F5" t="n">
-        <v>2</v>
-      </c>
-      <c r="G5" t="n">
-        <v>1</v>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>2026-07-30</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Global Defense, Inc. (100th pct, Deep Dive); Askari Defense, Inc. (50th pct, Pass); Mentat Biotechnology, Corp. (17th pct, Pass)</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/2144303/000214430326000001/0002144303-26-000001-index.htm; https://www.sec.gov/Archives/edgar/data/2037822/000203782226000003/0002037822-26-000003-index.htm; https://www.sec.gov/Archives/edgar/data/2133514/000101297526000649/0001012975-26-000649-index.htm; https://www.sec.gov/Archives/edgar/data/2128641/000101297526000648/0001012975-26-000648-index.htm</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>Emerging: technical signal running ahead of mainstream coverage.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>defense</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>defense, decimus, dover, select, security, aventura</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>12</v>
-      </c>
-      <c r="D6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E6" t="n">
-        <v>6</v>
-      </c>
-      <c r="F6" t="n">
-        <v>2</v>
-      </c>
-      <c r="G6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>Global Defense, Inc. (100th pct, Watch); Askari Defense, Inc. (50th pct, Pass); Mentat Biotechnology, Corp. (33th pct, Pass)</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/2144303/000214430326000001/0002144303-26-000001-index.htm; https://www.sec.gov/Archives/edgar/data/2037822/000203782226000003/0002037822-26-000003-index.htm; https://www.sec.gov/Archives/edgar/data/2133514/000101297526000649/0001012975-26-000649-index.htm; https://www.sec.gov/Archives/edgar/data/2128641/000101297526000648/0001012975-26-000648-index.htm</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>Emerging: technical signal running ahead of mainstream coverage.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>defense</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>defense, decimus, dover, select, security, aventura</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>12</v>
-      </c>
-      <c r="D7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E7" t="n">
-        <v>6</v>
-      </c>
-      <c r="F7" t="n">
-        <v>2</v>
-      </c>
-      <c r="G7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>Global Defense, Inc. (100th pct, Watch); Askari Defense, Inc. (50th pct, Pass)</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/Archives/edgar/data/2144303/000214430326000001/0002144303-26-000001-index.htm; https://www.sec.gov/Archives/edgar/data/2037822/000203782226000003/0002037822-26-000003-index.htm; https://www.sec.gov/Archives/edgar/data/2133514/000101297526000649/0001012975-26-000649-index.htm; https://www.sec.gov/Archives/edgar/data/2128641/000101297526000648/0001012975-26-000648-index.htm</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
         <is>
           <t>Emerging: technical signal running ahead of mainstream coverage.</t>
         </is>
@@ -7438,7 +7250,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7483,405 +7295,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>SpaceX Starship Flight 13 livestream [video]</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>hn</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>2026-07-24</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>[STUB: no API key — judgment unavailable] — matched thesis theme: Defence Tech</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>https://news.ycombinator.com/item?id=49042528</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>London Gatwick has launched a robotic airport parking service</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>hn</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>2026-07-26</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>[STUB: no API key — judgment unavailable] — matched thesis theme: Robotics &amp; Physical AI</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>https://news.ycombinator.com/item?id=49058669</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Xiaomi-Robotics-1</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>hn</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>[STUB: no API key — judgment unavailable] — matched thesis theme: Robotics &amp; Physical AI</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>https://news.ycombinator.com/item?id=48974454</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>San Francisco: Don't Fall for Industry Defense of Surveillance Pricing</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>hn</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>2026-07-29</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>[STUB: no API key — judgment unavailable] — matched thesis theme: Defence Tech</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>https://news.ycombinator.com/item?id=49096885</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Jensen Huang's first post on Twitter is in defense of open access to AI models</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>hn</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>2026-07-27</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>[STUB: no API key — judgment unavailable] — matched thesis theme: Defence Tech</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>https://news.ycombinator.com/item?id=49073267</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Robotics development made dead simple (open source)</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>hn</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>2026-07-26</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>[STUB: no API key — judgment unavailable] — matched thesis theme: Robotics &amp; Physical AI</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>https://news.ycombinator.com/item?id=49058956</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>US House passes $1T defense bill despite Iran, Israel concerns</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>hn</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>2026-07-23</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>[STUB: no API key — judgment unavailable] — matched thesis theme: Defence Tech</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>https://news.ycombinator.com/item?id=49023271</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>US House Narrowly Passes Controversial National Defense Authorization Act</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>hn</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>2026-07-22</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>[STUB: no API key — judgment unavailable] — matched thesis theme: Defence Tech</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>https://news.ycombinator.com/item?id=49014795</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>YouTube System Design for Robotics Data Infrastructure</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>hn</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>2026-07-21</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>[STUB: no API key — judgment unavailable] — matched thesis theme: Robotics &amp; Physical AI</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>https://news.ycombinator.com/item?id=48995923</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Tesla's profits slide despite growing revenue as it pivots to robotics and AI</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>hn</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>2026-07-22</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>[STUB: no API key — judgment unavailable] — matched thesis theme: Robotics &amp; Physical AI</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>https://news.ycombinator.com/item?id=49014549</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Securing America's Defense Supply Chains</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>hn</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>2026-07-21</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>[STUB: no API key — judgment unavailable] — matched thesis theme: Defence Tech</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>https://news.ycombinator.com/item?id=48994840</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>The Robots Cometh</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>hn</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>2026-07-24</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>[STUB: no API key — judgment unavailable] — matched thesis theme: Robotics &amp; Physical AI</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>https://news.ycombinator.com/item?id=49034436</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Ask HN: Anyone working on practical robotics (cobots) for the home?</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>hn</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>2026-07-22</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>[STUB: no API key — judgment unavailable] — matched thesis theme: Robotics &amp; Physical AI</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>https://news.ycombinator.com/item?id=49010573</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Claude Plays Robotics</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>hn</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>[STUB: no API key — judgment unavailable] — matched thesis theme: Robotics &amp; Physical AI</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>https://news.ycombinator.com/item?id=48980787</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>The Future of American Defense – Y Combinator [video]</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>hn</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>2026-07-26</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>[STUB: no API key — judgment unavailable] — matched thesis theme: Defence Tech</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>https://news.ycombinator.com/item?id=49056441</t>
+          <t>— curation pass has not run (or nothing met the bar since last digest)</t>
         </is>
       </c>
     </row>
@@ -9728,12 +9142,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Pentra Robotics, inc.</t>
+          <t>Vitanova Biomedical Inc.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>robotics</t>
+          <t>biotech_health</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -9743,11 +9157,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -9763,12 +9177,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Sielo Robotics Inc.</t>
+          <t>Mentat Biotechnology, Corp.</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>robotics</t>
+          <t>biotech_health</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -9778,11 +9192,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -9798,12 +9212,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Vitanova Biomedical Inc.</t>
+          <t>Venus Aerospace Corp.</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>biotech_health</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -9813,11 +9227,11 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -9833,12 +9247,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Mentat Biotechnology, Corp.</t>
+          <t>Sielo Robotics Inc.</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>biotech_health</t>
+          <t>robotics</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -9848,11 +9262,11 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -9868,12 +9282,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Venus Aerospace Corp.</t>
+          <t>Luminous Robotics, Inc.</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>robotics</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -9883,11 +9297,11 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -9903,17 +9317,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Luminous Robotics, Inc.</t>
+          <t>JuliaHub</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>robotics</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>series-b</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -9922,7 +9336,7 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -9938,26 +9352,26 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>JuliaHub</t>
+          <t>Pentra Robotics, inc.</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>robotics</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>series-b</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>

</xml_diff>